<commit_message>
Add {{ qa_stamp }} placeholder to Excel and Visio sample templates
Align the .xlsx and .vsdx samples with the .docx flow and the automated
stamping workflow: both now carry a {{ qa_stamp }} tag (Excel in a QA STATUS
STAMP block, Visio in a dedicated shape) that the server render swaps for
qaapproved.png / qarejected.png based on document state.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_gmp_template.xlsx
+++ b/sample_gmp_template.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -748,18 +748,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>QA STATUS STAMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Stamp</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>{{ qa_stamp }}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>This is a {{ 'CONTROLLED COPY' if is_active else 'OBSOLETE' }} document — printed copies are uncontrolled.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A18:D18"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A20:D20"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>